<commit_message>
v0.9 - test reel Cisco 3750 + dark mode + historique scanner + detection equipements
</commit_message>
<xml_diff>
--- a/devices.xlsx
+++ b/devices.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amira\ocp-network-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5AD6EC-F2B7-40ED-8F4F-211D88B8A290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0290518-AE8D-4200-9152-20B431927D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1886" yWindow="1886" windowWidth="18514" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10971" yWindow="1114" windowWidth="23229" windowHeight="10466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t>name</t>
   </si>
@@ -48,9 +48,6 @@
     <t>device_type</t>
   </si>
   <si>
-    <t>R1</t>
-  </si>
-  <si>
     <t>127.0.0.1</t>
   </si>
   <si>
@@ -67,6 +64,21 @@
   </si>
   <si>
     <t>R3</t>
+  </si>
+  <si>
+    <t>Sw1</t>
+  </si>
+  <si>
+    <t>192.168.56.2</t>
+  </si>
+  <si>
+    <t>adminjorf</t>
+  </si>
+  <si>
+    <t>@csdsij0rf</t>
+  </si>
+  <si>
+    <t>cisco_ios</t>
   </si>
 </sst>
 </file>
@@ -429,71 +441,71 @@
     </row>
     <row r="2" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2">
-        <v>5000</v>
+        <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C3" s="2">
         <v>5001</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="29.15" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2">
         <v>5002</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>